<commit_message>
Addition of two brake wear scenarios
Addition of a low brake wear scenario for EVs and high brake wear to account for the variability of brake wear found in the literature. Brake wear for EVs is believed to increase as a result of higher vehicle weight and decrease from the use of regenerative braking.
Two new scenarios model a 20% increase in brake wear and a 80% decrease.
</commit_message>
<xml_diff>
--- a/outputs/scenarios.xlsx
+++ b/outputs/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_University_of_Toronto\11_Health_Co-Benefits_CO2_Mitigation_Scenarios\03_FLAME-AQ\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A227B0C7-CB1A-454A-B76B-950666F011E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8673DCB2-6FD0-41A3-B1FA-7D1FC3DD78D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="22605" windowHeight="14625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="147">
   <si>
     <t>Scenario</t>
   </si>
@@ -434,6 +434,33 @@
   </si>
   <si>
     <t>NREL_elec_intermediate_no_coal</t>
+  </si>
+  <si>
+    <t>ZEV_all_NREL_intermediate_BW_high</t>
+  </si>
+  <si>
+    <t>brake_tire_emissions_modification</t>
+  </si>
+  <si>
+    <t>high_brake</t>
+  </si>
+  <si>
+    <t>ZEV_all_NREL_intermediate_BW_low</t>
+  </si>
+  <si>
+    <t>scen_ZEV_all_NREL_inter_BW_high</t>
+  </si>
+  <si>
+    <t>ZEV_All_NREL_intermediate_BW_high</t>
+  </si>
+  <si>
+    <t>low_brake</t>
+  </si>
+  <si>
+    <t>scen_ZEV_all_NREL_inter_BW_low</t>
+  </si>
+  <si>
+    <t>ZEV_All_NREL_intermediate_BW_low</t>
   </si>
 </sst>
 </file>
@@ -1329,7 +1356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D217"/>
+  <dimension ref="A1:D231"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -4374,6 +4401,202 @@
         <v>46</v>
       </c>
     </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A219" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A220" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A222" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A225" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B225" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C225" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D225" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A226" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B226" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C226" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D226" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A227" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B227" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C227" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D227" s="7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A228" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B228" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C228" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D228" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A229" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B229" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C229" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D229" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A230" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B230" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C230" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D230" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A231" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B231" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C231" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D231" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New scenario - Only EVs
Addition of a scenario with 100% EVs by 2020.
</commit_message>
<xml_diff>
--- a/outputs/scenarios.xlsx
+++ b/outputs/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_University_of_Toronto\11_Health_Co-Benefits_CO2_Mitigation_Scenarios\03_FLAME-AQ\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8673DCB2-6FD0-41A3-B1FA-7D1FC3DD78D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5583BFD5-D1D8-42D3-8C51-5E8E8CE6F575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6615" yWindow="780" windowWidth="20055" windowHeight="14625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="150">
   <si>
     <t>Scenario</t>
   </si>
@@ -461,6 +461,15 @@
   </si>
   <si>
     <t>ZEV_All_NREL_intermediate_BW_low</t>
+  </si>
+  <si>
+    <t>EV100_NREL_Intermediate</t>
+  </si>
+  <si>
+    <t>scen_EV100_NREL_Intermediate</t>
+  </si>
+  <si>
+    <t>Evs100</t>
   </si>
 </sst>
 </file>
@@ -1356,7 +1365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D231"/>
+  <dimension ref="A1:D237"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -4597,6 +4606,90 @@
         <v>144</v>
       </c>
     </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A232" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B232" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A233" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B233" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A234" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B234" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A235" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B235" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D235" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A236" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B236" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A237" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B237" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C237" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D237" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>